<commit_message>
feat(agent): add account-based activity logging system in LOG directory
</commit_message>
<xml_diff>
--- a/agent/templates/견적서 샘플.xlsx
+++ b/agent/templates/견적서 샘플.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\smart_quote_sys\product_selector\Quote_manage\기본자료\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\업무\agent\smart_quote_sys\smart_quote_sys\product_selector\agent\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8F0E2E-18DE-4C28-80CD-8AD993A850FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B051D7F-B227-4961-8E98-1927BF1DB73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -647,14 +647,14 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="178" fontId="10" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -663,29 +663,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="178" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -695,24 +696,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -1124,7 +1124,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="53"/>
@@ -1176,7 +1176,7 @@
       <c r="W2" s="1"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="67" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="53"/>
@@ -1207,7 +1207,7 @@
       <c r="W3" s="5"/>
     </row>
     <row r="4" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="67" t="s">
+      <c r="A4" s="68" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="53"/>
@@ -1425,7 +1425,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="5"/>
-      <c r="C12" s="68"/>
+      <c r="C12" s="65"/>
       <c r="D12" s="53"/>
       <c r="E12" s="53"/>
       <c r="F12" s="53"/>
@@ -1505,11 +1505,11 @@
       <c r="A15" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="69" t="s">
+      <c r="B15" s="54" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="60"/>
-      <c r="D15" s="69" t="s">
+      <c r="D15" s="54" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="60"/>
@@ -1520,10 +1520,10 @@
       <c r="H15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="69" t="s">
+      <c r="I15" s="54" t="s">
         <v>19</v>
       </c>
-      <c r="J15" s="61"/>
+      <c r="J15" s="55"/>
       <c r="K15" s="20"/>
       <c r="L15" s="20"/>
       <c r="M15" s="20"/>
@@ -1540,15 +1540,15 @@
     </row>
     <row r="16" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="21"/>
-      <c r="B16" s="72"/>
-      <c r="C16" s="73"/>
-      <c r="D16" s="74"/>
-      <c r="E16" s="75"/>
-      <c r="F16" s="75"/>
+      <c r="B16" s="61"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="63"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
       <c r="G16" s="22"/>
       <c r="H16" s="23"/>
-      <c r="I16" s="70"/>
-      <c r="J16" s="71"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="57"/>
       <c r="K16" s="24"/>
       <c r="L16" s="24"/>
       <c r="M16" s="24"/>
@@ -1565,15 +1565,15 @@
     </row>
     <row r="17" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25"/>
-      <c r="B17" s="48"/>
-      <c r="C17" s="49"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="47"/>
       <c r="D17" s="50"/>
       <c r="E17" s="51"/>
       <c r="F17" s="51"/>
       <c r="G17" s="26"/>
       <c r="H17" s="27"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="58"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="59"/>
       <c r="K17" s="24"/>
       <c r="L17" s="24"/>
       <c r="M17" s="24"/>
@@ -1590,15 +1590,15 @@
     </row>
     <row r="18" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="25"/>
-      <c r="B18" s="48"/>
-      <c r="C18" s="49"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="47"/>
       <c r="D18" s="50"/>
       <c r="E18" s="51"/>
       <c r="F18" s="51"/>
       <c r="G18" s="26"/>
       <c r="H18" s="28"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="58"/>
+      <c r="I18" s="58"/>
+      <c r="J18" s="59"/>
       <c r="K18" s="29"/>
       <c r="L18" s="30"/>
       <c r="M18" s="29"/>
@@ -1615,15 +1615,15 @@
     </row>
     <row r="19" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="25"/>
-      <c r="B19" s="48"/>
-      <c r="C19" s="49"/>
+      <c r="B19" s="46"/>
+      <c r="C19" s="47"/>
       <c r="D19" s="50"/>
       <c r="E19" s="51"/>
       <c r="F19" s="51"/>
       <c r="G19" s="31"/>
       <c r="H19" s="28"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="58"/>
+      <c r="I19" s="58"/>
+      <c r="J19" s="59"/>
       <c r="K19" s="24"/>
       <c r="L19" s="24"/>
       <c r="M19" s="24"/>
@@ -1640,15 +1640,15 @@
     </row>
     <row r="20" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
-      <c r="B20" s="48"/>
-      <c r="C20" s="49"/>
+      <c r="B20" s="46"/>
+      <c r="C20" s="47"/>
       <c r="D20" s="50"/>
       <c r="E20" s="51"/>
       <c r="F20" s="51"/>
       <c r="G20" s="31"/>
       <c r="H20" s="28"/>
-      <c r="I20" s="55"/>
-      <c r="J20" s="56"/>
+      <c r="I20" s="48"/>
+      <c r="J20" s="49"/>
       <c r="K20" s="24"/>
       <c r="L20" s="24"/>
       <c r="M20" s="24"/>
@@ -1665,15 +1665,15 @@
     </row>
     <row r="21" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="32"/>
-      <c r="B21" s="48"/>
-      <c r="C21" s="49"/>
+      <c r="B21" s="46"/>
+      <c r="C21" s="47"/>
       <c r="D21" s="50"/>
       <c r="E21" s="51"/>
       <c r="F21" s="51"/>
       <c r="G21" s="31"/>
       <c r="H21" s="28"/>
-      <c r="I21" s="55"/>
-      <c r="J21" s="56"/>
+      <c r="I21" s="48"/>
+      <c r="J21" s="49"/>
       <c r="K21" s="24"/>
       <c r="L21" s="24"/>
       <c r="M21" s="24"/>
@@ -1690,15 +1690,15 @@
     </row>
     <row r="22" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="32"/>
-      <c r="B22" s="48"/>
-      <c r="C22" s="49"/>
+      <c r="B22" s="46"/>
+      <c r="C22" s="47"/>
       <c r="D22" s="50"/>
       <c r="E22" s="51"/>
       <c r="F22" s="51"/>
       <c r="G22" s="31"/>
       <c r="H22" s="28"/>
-      <c r="I22" s="55"/>
-      <c r="J22" s="56"/>
+      <c r="I22" s="48"/>
+      <c r="J22" s="49"/>
       <c r="K22" s="24"/>
       <c r="L22" s="24"/>
       <c r="M22" s="24"/>
@@ -1715,15 +1715,15 @@
     </row>
     <row r="23" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="32"/>
-      <c r="B23" s="48"/>
-      <c r="C23" s="49"/>
+      <c r="B23" s="46"/>
+      <c r="C23" s="47"/>
       <c r="D23" s="50"/>
       <c r="E23" s="51"/>
       <c r="F23" s="51"/>
       <c r="G23" s="31"/>
       <c r="H23" s="28"/>
-      <c r="I23" s="55"/>
-      <c r="J23" s="56"/>
+      <c r="I23" s="48"/>
+      <c r="J23" s="49"/>
       <c r="K23" s="24"/>
       <c r="L23" s="24"/>
       <c r="M23" s="24"/>
@@ -1740,15 +1740,15 @@
     </row>
     <row r="24" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="32"/>
-      <c r="B24" s="48"/>
-      <c r="C24" s="49"/>
+      <c r="B24" s="46"/>
+      <c r="C24" s="47"/>
       <c r="D24" s="50"/>
       <c r="E24" s="51"/>
       <c r="F24" s="51"/>
       <c r="G24" s="31"/>
       <c r="H24" s="28"/>
-      <c r="I24" s="55"/>
-      <c r="J24" s="56"/>
+      <c r="I24" s="48"/>
+      <c r="J24" s="49"/>
       <c r="K24" s="24"/>
       <c r="L24" s="24"/>
       <c r="M24" s="24"/>
@@ -1765,15 +1765,15 @@
     </row>
     <row r="25" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="32"/>
-      <c r="B25" s="48"/>
-      <c r="C25" s="49"/>
+      <c r="B25" s="46"/>
+      <c r="C25" s="47"/>
       <c r="D25" s="50"/>
       <c r="E25" s="51"/>
       <c r="F25" s="51"/>
       <c r="G25" s="31"/>
       <c r="H25" s="28"/>
-      <c r="I25" s="55"/>
-      <c r="J25" s="56"/>
+      <c r="I25" s="48"/>
+      <c r="J25" s="49"/>
       <c r="K25" s="24"/>
       <c r="L25" s="24"/>
       <c r="M25" s="24"/>
@@ -1790,15 +1790,15 @@
     </row>
     <row r="26" spans="1:23" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="33"/>
-      <c r="B26" s="48"/>
-      <c r="C26" s="49"/>
+      <c r="B26" s="46"/>
+      <c r="C26" s="47"/>
       <c r="D26" s="50"/>
       <c r="E26" s="51"/>
       <c r="F26" s="51"/>
       <c r="G26" s="31"/>
       <c r="H26" s="28"/>
-      <c r="I26" s="55"/>
-      <c r="J26" s="56"/>
+      <c r="I26" s="48"/>
+      <c r="J26" s="49"/>
       <c r="K26" s="24"/>
       <c r="L26" s="24"/>
       <c r="M26" s="24"/>
@@ -1815,15 +1815,15 @@
     </row>
     <row r="27" spans="1:23" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="32"/>
-      <c r="B27" s="48"/>
-      <c r="C27" s="49"/>
+      <c r="B27" s="46"/>
+      <c r="C27" s="47"/>
       <c r="D27" s="50"/>
       <c r="E27" s="51"/>
       <c r="F27" s="51"/>
       <c r="G27" s="31"/>
       <c r="H27" s="28"/>
-      <c r="I27" s="55"/>
-      <c r="J27" s="56"/>
+      <c r="I27" s="48"/>
+      <c r="J27" s="49"/>
       <c r="K27" s="24"/>
       <c r="L27" s="24"/>
       <c r="M27" s="24"/>
@@ -1840,15 +1840,15 @@
     </row>
     <row r="28" spans="1:23" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="32"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="49"/>
+      <c r="B28" s="46"/>
+      <c r="C28" s="47"/>
       <c r="D28" s="50"/>
       <c r="E28" s="51"/>
       <c r="F28" s="51"/>
       <c r="G28" s="31"/>
       <c r="H28" s="28"/>
-      <c r="I28" s="55"/>
-      <c r="J28" s="56"/>
+      <c r="I28" s="48"/>
+      <c r="J28" s="49"/>
       <c r="K28" s="24"/>
       <c r="L28" s="24"/>
       <c r="M28" s="24"/>
@@ -1865,15 +1865,15 @@
     </row>
     <row r="29" spans="1:23" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="34"/>
-      <c r="B29" s="63"/>
-      <c r="C29" s="64"/>
-      <c r="D29" s="46"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
+      <c r="B29" s="72"/>
+      <c r="C29" s="73"/>
+      <c r="D29" s="74"/>
+      <c r="E29" s="75"/>
+      <c r="F29" s="75"/>
       <c r="G29" s="35"/>
       <c r="H29" s="36"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="58"/>
+      <c r="I29" s="58"/>
+      <c r="J29" s="59"/>
       <c r="K29" s="24"/>
       <c r="L29" s="24"/>
       <c r="M29" s="24"/>
@@ -1889,7 +1889,7 @@
       <c r="W29" s="24"/>
     </row>
     <row r="30" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="59"/>
+      <c r="A30" s="70"/>
       <c r="B30" s="60"/>
       <c r="C30" s="60"/>
       <c r="D30" s="60"/>
@@ -1898,7 +1898,7 @@
       <c r="G30" s="60"/>
       <c r="H30" s="60"/>
       <c r="I30" s="60"/>
-      <c r="J30" s="61"/>
+      <c r="J30" s="55"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -1992,7 +1992,7 @@
       <c r="A34" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="62"/>
+      <c r="B34" s="71"/>
       <c r="C34" s="53"/>
       <c r="D34" s="53"/>
       <c r="E34" s="53"/>
@@ -2023,7 +2023,7 @@
       <c r="E35" s="53"/>
       <c r="F35" s="53"/>
       <c r="G35" s="45"/>
-      <c r="H35" s="54"/>
+      <c r="H35" s="69"/>
       <c r="I35" s="53"/>
       <c r="J35" s="53"/>
       <c r="K35" s="1"/>
@@ -2048,7 +2048,7 @@
       <c r="E36" s="53"/>
       <c r="F36" s="53"/>
       <c r="G36" s="45"/>
-      <c r="H36" s="54"/>
+      <c r="H36" s="69"/>
       <c r="I36" s="53"/>
       <c r="J36" s="53"/>
       <c r="K36" s="1"/>
@@ -2154,7 +2154,7 @@
       <c r="E40" s="53"/>
       <c r="F40" s="53"/>
       <c r="G40" s="45"/>
-      <c r="H40" s="54"/>
+      <c r="H40" s="69"/>
       <c r="I40" s="53"/>
       <c r="J40" s="53"/>
       <c r="K40" s="1"/>
@@ -2179,7 +2179,7 @@
       <c r="E41" s="1"/>
       <c r="F41" s="3"/>
       <c r="G41" s="45"/>
-      <c r="H41" s="54"/>
+      <c r="H41" s="69"/>
       <c r="I41" s="53"/>
       <c r="J41" s="53"/>
       <c r="K41" s="1"/>
@@ -2204,7 +2204,7 @@
       <c r="E42" s="1"/>
       <c r="F42" s="3"/>
       <c r="G42" s="45"/>
-      <c r="H42" s="54"/>
+      <c r="H42" s="69"/>
       <c r="I42" s="53"/>
       <c r="J42" s="53"/>
       <c r="K42" s="1"/>
@@ -26223,14 +26223,51 @@
     </row>
   </sheetData>
   <mergeCells count="69">
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="I25:J25"/>
-    <mergeCell ref="I26:J26"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I24:J24"/>
+    <mergeCell ref="D29:F29"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="I28:J28"/>
+    <mergeCell ref="I29:J29"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="D28:F28"/>
+    <mergeCell ref="B34:F40"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C13:F13"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="D19:F19"/>
@@ -26247,56 +26284,19 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:F16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H39:J39"/>
-    <mergeCell ref="H40:J40"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I28:J28"/>
-    <mergeCell ref="I29:J29"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="H37:J37"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="A30:J30"/>
-    <mergeCell ref="D27:F27"/>
-    <mergeCell ref="D28:F28"/>
-    <mergeCell ref="B34:F40"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="D29:F29"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="I25:J25"/>
+    <mergeCell ref="I26:J26"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I24:J24"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0" right="0" top="0.59055118110236215" bottom="0" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="76" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="60" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>